<commit_message>
Add report history with PDF and Excel export
</commit_message>
<xml_diff>
--- a/backend/reports/AI_Review_Report.xlsx
+++ b/backend/reports/AI_Review_Report.xlsx
@@ -439,7 +439,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>18</v>
+        <v>9</v>
       </c>
     </row>
     <row r="4">
@@ -449,7 +449,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
     </row>
     <row r="5">
@@ -459,7 +459,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="6">
@@ -469,7 +469,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
     </row>
     <row r="7">
@@ -479,7 +479,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>4.11</v>
+        <v>3.56</v>
       </c>
     </row>
     <row r="8">
@@ -490,7 +490,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>77.11%</t>
+          <t>84.04%</t>
         </is>
       </c>
     </row>

</xml_diff>